<commit_message>
docs(arquitectura): ADR con patrones, drivers medibles, modelo alineado, matrices, convenciones por stack y CI (#1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/matrices/Colaboraciones y responsabilidades.xlsx
+++ b/seguimiento/matrices/Colaboraciones y responsabilidades.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Crear la cuenta; valida correo unico, edad minima y contrasena.</t>
+          <t>Crear la cuenta; valida correo unico, edad minima, contrasena y consentimiento de datos.</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Dejar ese canal por defecto para el resto de la conversacion.</t>
+          <t>Saber por que canal llego cada mensaje para entregar la traduccion por el mismo.</t>
         </is>
       </c>
     </row>
@@ -963,6 +963,50 @@
       <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Ubicar la region dentro de un pais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Usuario</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Eliminar la cuenta</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Conversacion, MensajeOriginal, MensajeDestino</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Borrar la cuenta con todos sus datos (derecho al olvido).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Lenguaje</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Relacionarse con sus regiones</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Region (LenguajeRegion)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Saber en que regiones se habla cada idioma para validar Conversacion-RN-1.</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1044,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Falta validar con Farid si Reporte debe ser una entidad propia (hoy es una responsabilidad de Lenguaje).</t>
+          <t>Reporte queda como tabla de soporte (ADR-008), no como objeto de dominio.</t>
         </is>
       </c>
     </row>

</xml_diff>